<commit_message>
feat: import excel for add bulk employee
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
+++ b/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\WORK\simdatuk-dev\storage\app\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\WORK\simdatuk-dev\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -13,8 +13,8 @@
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
-    <sheet name="Pendidikan" sheetId="2" r:id="rId2"/>
-    <sheet name="Catatan" sheetId="15" r:id="rId3"/>
+    <sheet name="Riwayat Pendidikan" sheetId="2" r:id="rId2"/>
+    <sheet name="Riwayat Catatan" sheetId="15" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -25,32 +25,47 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Windows User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+* Masukkan Jabatan dari Hirarki tertinggi
+* Pisahkan Hirarki menggunakan tanda '&gt;'
+Contoh 1 : Misal Jabatan 'Arsiparis'
+Kepala Sekretariat Wakil Presiden&gt;Deputi Bidang Administrasi&gt;Kepala Biro Umum&gt;Arsiparis
+Contoh 2 : Misal Jabatan 'Staf Khusus Wakil Presiden (Bidang Umum)'
+Staf Khusus Wakil Presiden&gt;Staf Khusus Wakil Presiden (Bidang Umum)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
-  <si>
-    <t>Nama</t>
-  </si>
-  <si>
-    <t>Golongan</t>
-  </si>
-  <si>
-    <t>NIP</t>
-  </si>
-  <si>
-    <t>NRP</t>
-  </si>
-  <si>
-    <t>Tempat Lahir</t>
-  </si>
-  <si>
-    <t>Agama</t>
-  </si>
-  <si>
-    <t>Tingkat</t>
-  </si>
-  <si>
-    <t>Nama Sekolah</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Fakultas</t>
   </si>
@@ -58,66 +73,9 @@
     <t>Jurusan</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Tahun Lulus</t>
-  </si>
-  <si>
-    <t>TMT Golongan</t>
-  </si>
-  <si>
-    <t>Tanggal Lahir</t>
-  </si>
-  <si>
-    <t>Nama Gelar Depan</t>
-  </si>
-  <si>
-    <t>Nama Gelar Belakang</t>
-  </si>
-  <si>
-    <t>Jenis Kelamin</t>
-  </si>
-  <si>
-    <t>Status Perkawinan</t>
-  </si>
-  <si>
-    <t>Jenis Pegawai</t>
-  </si>
-  <si>
-    <t>Jenis Outsourcing</t>
-  </si>
-  <si>
-    <t>Eselon</t>
-  </si>
-  <si>
-    <t>TMT Eselon</t>
-  </si>
-  <si>
-    <t>Instansi Induk</t>
-  </si>
-  <si>
-    <t>Nama Sekolah/Universitas</t>
-  </si>
-  <si>
-    <t>No Karpeg</t>
-  </si>
-  <si>
     <t>NPWP</t>
   </si>
   <si>
-    <t>Status Pegawai</t>
-  </si>
-  <si>
-    <t>No KK</t>
-  </si>
-  <si>
-    <t>No NIK</t>
-  </si>
-  <si>
-    <t>Komplek</t>
-  </si>
-  <si>
     <t>Alamat Tempat Tinggal Saat Ini</t>
   </si>
   <si>
@@ -136,26 +94,92 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai)</t>
-  </si>
-  <si>
     <t>Keterangan Sekolah</t>
   </si>
   <si>
-    <t>Catatan</t>
-  </si>
-  <si>
-    <t>NIK</t>
-  </si>
-  <si>
-    <t>No Karisu</t>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t>NIK *</t>
+  </si>
+  <si>
+    <t>Nama *</t>
+  </si>
+  <si>
+    <t>NIP *</t>
+  </si>
+  <si>
+    <t>Tempat Lahir *</t>
+  </si>
+  <si>
+    <t>Tanggal Lahir *</t>
+  </si>
+  <si>
+    <t>Agama *</t>
+  </si>
+  <si>
+    <t>Jenis Kelamin *</t>
+  </si>
+  <si>
+    <t>Status Perkawinan *</t>
+  </si>
+  <si>
+    <t>Tingkat *</t>
+  </si>
+  <si>
+    <t>Nama Sekolah/Universitas *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tahun Lulus * </t>
+  </si>
+  <si>
+    <t>Status Pegawai *</t>
+  </si>
+  <si>
+    <t>No NIK *</t>
+  </si>
+  <si>
+    <t>Komplek *</t>
+  </si>
+  <si>
+    <t>Nama Sekolah *</t>
+  </si>
+  <si>
+    <t>Status *</t>
+  </si>
+  <si>
+    <t>Tahun Lulus *</t>
+  </si>
+  <si>
+    <t>Catatan *</t>
+  </si>
+  <si>
+    <t>Jabatan *</t>
+  </si>
+  <si>
+    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai) *</t>
+  </si>
+  <si>
+    <t>No KK *</t>
+  </si>
+  <si>
+    <t>Tingkat Pendidikan Terakhir*</t>
+  </si>
+  <si>
+    <t>Jenis Outsourcing *</t>
+  </si>
+  <si>
+    <t>Tanggal Mulai Bekerja *</t>
+  </si>
+  <si>
+    <t>TMT Menjabat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,6 +202,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -488,159 +525,132 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.5703125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="33.140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="24" style="1" customWidth="1"/>
-    <col min="19" max="19" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="67" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="25.28515625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="19.28515625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="67" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="25.28515625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="P1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="X1" s="2" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AC1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>36</v>
-      </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="AG2" s="3"/>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="AG3" s="3"/>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -653,37 +663,37 @@
     <col min="2" max="2" width="22.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -704,10 +714,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(Feat-B-005): Import Employees new mandatory field and field changes #2
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
+++ b/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
@@ -9,12 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
-    <sheet name="Riwayat Pendidikan" sheetId="2" r:id="rId2"/>
-    <sheet name="Riwayat Catatan" sheetId="15" r:id="rId3"/>
+    <sheet name="Riwayat Jabatan" sheetId="17" r:id="rId2"/>
+    <sheet name="Riwayat Pelatihan Teknis" sheetId="18" r:id="rId3"/>
     <sheet name="Riwayat Keluarga" sheetId="16" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
@@ -242,17 +242,17 @@
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Tingkat</t>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
         </r>
         <r>
           <rPr>
@@ -262,28 +262,32 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-- SD/Sederajat
-- SLTP/Sederajat
-- SLTA/Sederajat
-- Diploma I/II
-- Akademik/D3/S.Muda
-- Diploma IV/Strata I
-- Strata II
-- Strata III</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Status</t>
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenjang Jabatan</t>
         </r>
         <r>
           <rPr>
@@ -293,11 +297,39 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-- Lulus
-- DO
-- Aktif
-- Non-aktif
-- Mengundurkan Diri</t>
+- Eselon I
+- Eselon II
+- Eselon III
+- Fungsional
+- Pelaksana
+- Staf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Keterangan Jabatan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Promosi
+- Mutasi
+- Inpassing
+- Konversi</t>
         </r>
       </text>
     </comment>
@@ -306,6 +338,51 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
@@ -464,13 +541,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="47">
-  <si>
-    <t>Fakultas</t>
-  </si>
-  <si>
-    <t>Jurusan</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
   <si>
     <t>NPWP</t>
   </si>
@@ -490,9 +561,6 @@
     <t>No Telepon Kantor</t>
   </si>
   <si>
-    <t>Keterangan Sekolah</t>
-  </si>
-  <si>
     <t>Keterangan</t>
   </si>
   <si>
@@ -520,24 +588,9 @@
     <t>Status Perkawinan *</t>
   </si>
   <si>
-    <t>Tingkat *</t>
-  </si>
-  <si>
     <t>No NIK *</t>
   </si>
   <si>
-    <t>Nama Sekolah *</t>
-  </si>
-  <si>
-    <t>Status *</t>
-  </si>
-  <si>
-    <t>Tahun Lulus *</t>
-  </si>
-  <si>
-    <t>Catatan *</t>
-  </si>
-  <si>
     <t>Jabatan *</t>
   </si>
   <si>
@@ -605,6 +658,63 @@
   </si>
   <si>
     <t>Urut Keluarga</t>
+  </si>
+  <si>
+    <t>Nama Riwayat Jabatan *</t>
+  </si>
+  <si>
+    <t>Bulan Periode Input Riwayat *</t>
+  </si>
+  <si>
+    <t>Tahun Periode Input Riwayat *</t>
+  </si>
+  <si>
+    <t>Rumpun</t>
+  </si>
+  <si>
+    <t>Jenjang Jabatan</t>
+  </si>
+  <si>
+    <t>Keterangan Jabatan</t>
+  </si>
+  <si>
+    <t>SK Jabatan</t>
+  </si>
+  <si>
+    <t>Jenis SK Jabatan</t>
+  </si>
+  <si>
+    <t>No SK Jabatan</t>
+  </si>
+  <si>
+    <t>Tanggal SK Jabatan</t>
+  </si>
+  <si>
+    <t>TMT Selesai</t>
+  </si>
+  <si>
+    <t>SK Selesai</t>
+  </si>
+  <si>
+    <t>Jenis SK Selesai</t>
+  </si>
+  <si>
+    <t>No SK Selesai</t>
+  </si>
+  <si>
+    <t>Tanggal SK Selesai</t>
+  </si>
+  <si>
+    <t>Nama Diklat *</t>
+  </si>
+  <si>
+    <t>No Surat Perintah *</t>
+  </si>
+  <si>
+    <t>Tanggal Pelaksanaan *</t>
+  </si>
+  <si>
+    <t>Durasi Pelatihan (Hari)</t>
   </si>
 </sst>
 </file>
@@ -1005,85 +1115,85 @@
   <sheetData>
     <row r="1" spans="1:27" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="S1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="U1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1096,81 +1206,120 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>8</v>
+        <v>44</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>23</v>
+        <v>41</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1182,7 +1331,8 @@
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
@@ -1192,58 +1342,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(Feat-B-043): add educations and notes to outsource
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
+++ b/public/template_excel/DATA PEGAWAI OUTSOURCE.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api\public\template_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\WORK\simdatuk-dev\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6739B93E-3C73-49DA-9042-771AE3FAF194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
-    <sheet name="Riwayat Jabatan" sheetId="17" r:id="rId2"/>
-    <sheet name="Riwayat Pelatihan Teknis" sheetId="18" r:id="rId3"/>
-    <sheet name="Riwayat Keluarga" sheetId="16" r:id="rId4"/>
+    <sheet name="Riwayat Pendidikan" sheetId="19" r:id="rId2"/>
+    <sheet name="Riwayat Jabatan" sheetId="17" r:id="rId3"/>
+    <sheet name="Riwayat Pelatihan Teknis" sheetId="18" r:id="rId4"/>
+    <sheet name="Riwayat Keluarga" sheetId="16" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="20" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -28,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -62,7 +63,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -87,7 +88,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -115,7 +116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -140,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -170,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -201,7 +202,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -238,12 +239,78 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tingkat</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- SD/Sederajat
+- SLTP/Sederajat
+- SLTA/Sederajat
+- Diploma I/II
+- Akademik/D3/S.Muda
+- Diploma IV/Strata I
+- Strata II
+- Strata III</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Wilayah</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Dalam Negeri
+- Luar Negeri</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -278,7 +345,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -307,7 +374,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -338,13 +405,13 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -379,7 +446,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -439,13 +506,13 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -470,7 +537,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -499,7 +566,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -533,7 +600,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -566,7 +633,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -598,7 +665,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="76">
   <si>
     <t>NPWP</t>
   </si>
@@ -802,12 +869,36 @@
   </si>
   <si>
     <t xml:space="preserve">Status Perkawinan </t>
+  </si>
+  <si>
+    <t>Tingkat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Sekolah </t>
+  </si>
+  <si>
+    <t>Wilayah</t>
+  </si>
+  <si>
+    <t>Akreditasi</t>
+  </si>
+  <si>
+    <t>Fakultas</t>
+  </si>
+  <si>
+    <t>Jurusan</t>
+  </si>
+  <si>
+    <t>Keterangan Sekolah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catatan </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1157,50 +1248,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="30.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="19.33203125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.5546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="58.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="33.109375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="30.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="19.28515625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="21.5703125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="33.140625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="75.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="58.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="75.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="67" style="1" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="7.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="25.33203125" style="1" customWidth="1"/>
-    <col min="40" max="40" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="16384" width="9.109375" style="1"/>
+    <col min="35" max="35" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="25.28515625" style="1" customWidth="1"/>
+    <col min="40" max="40" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -1283,7 +1374,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1292,84 +1383,44 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>41</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1379,23 +1430,30 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>51</v>
@@ -1404,28 +1462,52 @@
         <v>52</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>17</v>
+        <v>33</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1435,88 +1517,165 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.44140625" customWidth="1"/>
-    <col min="19" max="19" width="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" customWidth="1"/>
+    <col min="19" max="19" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>